<commit_message>
Integrate LaSecre Logo and Airtable for permanent ticket storage
</commit_message>
<xml_diff>
--- a/tmp/resum_lasecre_Q1_2026.xlsx
+++ b/tmp/resum_lasecre_Q1_2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="32">
   <si>
     <t>Data Registre</t>
   </si>
@@ -25,12 +25,15 @@
     <t>Import Total</t>
   </si>
   <si>
-    <t>IVA Estimat</t>
+    <t>Quota_IVA</t>
   </si>
   <si>
     <t>Categoria</t>
   </si>
   <si>
+    <t>Enllaç Foto</t>
+  </si>
+  <si>
     <t>25/3/2026 17:11:44</t>
   </si>
   <si>
@@ -43,6 +46,9 @@
     <t>Materials i Manteniment</t>
   </si>
   <si>
+    <t>1186483666723350</t>
+  </si>
+  <si>
     <t>25/3/2026 17:11:59</t>
   </si>
   <si>
@@ -52,6 +58,9 @@
     <t>Material i eines</t>
   </si>
   <si>
+    <t>2175320363209282</t>
+  </si>
+  <si>
     <t>25/3/2026 17:13:35</t>
   </si>
   <si>
@@ -61,6 +70,9 @@
     <t>Subministraments i manteniment</t>
   </si>
   <si>
+    <t>938905085798313</t>
+  </si>
+  <si>
     <t>25/3/2026 17:42:30</t>
   </si>
   <si>
@@ -70,7 +82,31 @@
     <t>Materials i Subministraments</t>
   </si>
   <si>
+    <t>1650500949418797</t>
+  </si>
+  <si>
     <t>Ferreteria Jaime Valls, C.B.</t>
+  </si>
+  <si>
+    <t>920645867253634</t>
+  </si>
+  <si>
+    <t>25/3/2026 18:42:56</t>
+  </si>
+  <si>
+    <t>Subministraments i eines</t>
+  </si>
+  <si>
+    <t>https://graph.facebook.com/v17.0/1675473236800047</t>
+  </si>
+  <si>
+    <t>25/3/2026 18:51:43</t>
+  </si>
+  <si>
+    <t>Ferreterías Jaime Valls, C.B.</t>
+  </si>
+  <si>
+    <t>https://graph.facebook.com/v17.0/1158254969651778</t>
   </si>
 </sst>
 </file>
@@ -456,7 +492,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -464,9 +500,10 @@
     <col min="3" max="3" width="25" customWidth="1"/>
     <col min="4" max="5" width="15" customWidth="1"/>
     <col min="6" max="6" width="20" customWidth="1"/>
+    <col min="7" max="7" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -485,16 +522,19 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D2">
         <v>32.59</v>
@@ -503,18 +543,21 @@
         <v>5.66</v>
       </c>
       <c r="F2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+      <c r="G2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D3">
         <v>32.59</v>
@@ -523,18 +566,21 @@
         <v>5.66</v>
       </c>
       <c r="F3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+      <c r="G3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D4">
         <v>32.59</v>
@@ -543,18 +589,21 @@
         <v>5.66</v>
       </c>
       <c r="F4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+      <c r="G4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B5" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D5">
         <v>32.59</v>
@@ -563,18 +612,21 @@
         <v>5.66</v>
       </c>
       <c r="F5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+      <c r="G5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C6" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="D6">
         <v>32.59</v>
@@ -583,7 +635,56 @@
         <v>5.66</v>
       </c>
       <c r="F6" t="s">
-        <v>15</v>
+        <v>18</v>
+      </c>
+      <c r="G6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7">
+        <v>32.59</v>
+      </c>
+      <c r="E7">
+        <v>5.66</v>
+      </c>
+      <c r="F7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8">
+        <v>32.59</v>
+      </c>
+      <c r="E8">
+        <v>5.66</v>
+      </c>
+      <c r="F8" t="s">
+        <v>27</v>
+      </c>
+      <c r="G8" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: New realistic branding, Effiguard number update, and Airtable-based Excel export
</commit_message>
<xml_diff>
--- a/tmp/resum_lasecre_Q1_2026.xlsx
+++ b/tmp/resum_lasecre_Q1_2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Data Registre</t>
   </si>
@@ -34,95 +34,32 @@
     <t>Enllaç Foto</t>
   </si>
   <si>
-    <t>25/3/2026 17:11:44</t>
-  </si>
-  <si>
-    <t>17/10/2023</t>
-  </si>
-  <si>
-    <t>Ferretería Jaime Valls, C.B.</t>
-  </si>
-  <si>
-    <t>Materials i Manteniment</t>
-  </si>
-  <si>
-    <t>1186483666723350</t>
-  </si>
-  <si>
-    <t>25/3/2026 17:11:59</t>
-  </si>
-  <si>
-    <t>Ferretería Jaime Valls</t>
-  </si>
-  <si>
-    <t>Material i eines</t>
-  </si>
-  <si>
-    <t>2175320363209282</t>
-  </si>
-  <si>
-    <t>25/3/2026 17:13:35</t>
-  </si>
-  <si>
-    <t>Jaime Valls, C.B. (Ferreteria)</t>
-  </si>
-  <si>
-    <t>Subministraments i manteniment</t>
-  </si>
-  <si>
-    <t>938905085798313</t>
-  </si>
-  <si>
-    <t>25/3/2026 17:42:30</t>
-  </si>
-  <si>
-    <t>Ferreteria Jaime Valls</t>
-  </si>
-  <si>
-    <t>Materials i Subministraments</t>
-  </si>
-  <si>
-    <t>1650500949418797</t>
-  </si>
-  <si>
-    <t>Ferreteria Jaime Valls, C.B.</t>
-  </si>
-  <si>
-    <t>920645867253634</t>
-  </si>
-  <si>
-    <t>25/3/2026 18:42:56</t>
-  </si>
-  <si>
-    <t>Subministraments i eines</t>
-  </si>
-  <si>
-    <t>https://graph.facebook.com/v17.0/1675473236800047</t>
-  </si>
-  <si>
-    <t>25/3/2026 18:51:43</t>
-  </si>
-  <si>
-    <t>Ferreterías Jaime Valls, C.B.</t>
-  </si>
-  <si>
-    <t>https://graph.facebook.com/v17.0/1158254969651778</t>
+    <t>27/3/2026 17:31:05</t>
+  </si>
+  <si>
+    <t>27/03/2026</t>
+  </si>
+  <si>
+    <t>Test Supermarket</t>
+  </si>
+  <si>
+    <t>Food &amp; Dining</t>
+  </si>
+  <si>
+    <t/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
       <scheme val="minor"/>
       <sz val="11"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
     </font>
   </fonts>
   <fills count="3">
@@ -152,7 +89,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -492,7 +429,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -537,154 +474,16 @@
         <v>9</v>
       </c>
       <c r="D2">
-        <v>32.59</v>
+        <v>42.5</v>
       </c>
       <c r="E2">
-        <v>5.66</v>
+        <v>8.5</v>
       </c>
       <c r="F2" t="s">
         <v>10</v>
       </c>
       <c r="G2" t="s">
         <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3">
-        <v>32.59</v>
-      </c>
-      <c r="E3">
-        <v>5.66</v>
-      </c>
-      <c r="F3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4">
-        <v>32.59</v>
-      </c>
-      <c r="E4">
-        <v>5.66</v>
-      </c>
-      <c r="F4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5">
-        <v>32.59</v>
-      </c>
-      <c r="E5">
-        <v>5.66</v>
-      </c>
-      <c r="F5" t="s">
-        <v>22</v>
-      </c>
-      <c r="G5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" t="s">
-        <v>24</v>
-      </c>
-      <c r="D6">
-        <v>32.59</v>
-      </c>
-      <c r="E6">
-        <v>5.66</v>
-      </c>
-      <c r="F6" t="s">
-        <v>18</v>
-      </c>
-      <c r="G6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>26</v>
-      </c>
-      <c r="B7" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D7">
-        <v>32.59</v>
-      </c>
-      <c r="E7">
-        <v>5.66</v>
-      </c>
-      <c r="F7" t="s">
-        <v>27</v>
-      </c>
-      <c r="G7" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" t="s">
-        <v>30</v>
-      </c>
-      <c r="D8">
-        <v>32.59</v>
-      </c>
-      <c r="E8">
-        <v>5.66</v>
-      </c>
-      <c r="F8" t="s">
-        <v>27</v>
-      </c>
-      <c r="G8" t="s">
-        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>